<commit_message>
Daily recap, matchup updates, learning and research 2026-08-10
</commit_message>
<xml_diff>
--- a/data/k-props/2026-08-10.xlsx
+++ b/data/k-props/2026-08-10.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="86">
   <si>
     <t>date</t>
   </si>
@@ -148,6 +148,9 @@
     <t>Sonny Gray</t>
   </si>
   <si>
+    <t>U</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
@@ -172,6 +175,12 @@
     <t>Christian Scott</t>
   </si>
   <si>
+    <t>O</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
     <t>6-7</t>
   </si>
   <si>
@@ -179,6 +188,9 @@
   </si>
   <si>
     <t>Bryce Elder</t>
+  </si>
+  <si>
+    <t>L</t>
   </si>
   <si>
     <t>Trevor Rogers</t>
@@ -793,26 +805,32 @@
       <c r="F2">
         <v>4.5</v>
       </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
       <c r="H2" t="s">
         <v>45</v>
       </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
       <c r="J2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K2">
         <v>4.5</v>
       </c>
       <c r="L2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="N2">
         <v>822780</v>
       </c>
       <c r="O2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P2">
         <v>5.7</v>
@@ -854,7 +872,7 @@
         <v>0.9895</v>
       </c>
       <c r="AC2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD2">
         <v>0.2201</v>
@@ -878,13 +896,25 @@
         <v>1</v>
       </c>
       <c r="AK2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AM2">
         <v>0</v>
+      </c>
+      <c r="AN2">
+        <v>-0.5</v>
+      </c>
+      <c r="AO2">
+        <v>0.5</v>
+      </c>
+      <c r="AP2">
+        <v>-0.5</v>
+      </c>
+      <c r="AQ2">
+        <v>0.5</v>
       </c>
     </row>
     <row r="3" spans="1:43" x14ac:dyDescent="0.25">
@@ -892,7 +922,7 @@
         <v>43</v>
       </c>
       <c r="B3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C3">
         <v>4.5</v>
@@ -906,26 +936,32 @@
       <c r="F3">
         <v>4.17</v>
       </c>
+      <c r="G3">
+        <v>3</v>
+      </c>
       <c r="H3" t="s">
         <v>45</v>
       </c>
+      <c r="I3">
+        <v>-0.33</v>
+      </c>
       <c r="J3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K3">
         <v>4.17</v>
       </c>
       <c r="L3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="N3">
         <v>822780</v>
       </c>
       <c r="O3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P3">
         <v>5</v>
@@ -967,7 +1003,7 @@
         <v>0.8849</v>
       </c>
       <c r="AC3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD3">
         <v>0.1968</v>
@@ -991,13 +1027,25 @@
         <v>1</v>
       </c>
       <c r="AK3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AM3">
         <v>0</v>
+      </c>
+      <c r="AN3">
+        <v>-1.17</v>
+      </c>
+      <c r="AO3">
+        <v>1.17</v>
+      </c>
+      <c r="AP3">
+        <v>-1.17</v>
+      </c>
+      <c r="AQ3">
+        <v>1.17</v>
       </c>
     </row>
     <row r="4" spans="1:43" x14ac:dyDescent="0.25">
@@ -1005,7 +1053,7 @@
         <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C4">
         <v>5.5</v>
@@ -1019,26 +1067,32 @@
       <c r="F4">
         <v>6.61</v>
       </c>
+      <c r="G4">
+        <v>6</v>
+      </c>
       <c r="H4" t="s">
-        <v>45</v>
+        <v>54</v>
+      </c>
+      <c r="I4">
+        <v>1.11</v>
       </c>
       <c r="J4" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="K4">
         <v>6.61</v>
       </c>
       <c r="L4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="M4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="N4">
         <v>824887</v>
       </c>
       <c r="O4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P4">
         <v>4.6</v>
@@ -1080,7 +1134,7 @@
         <v>1.0853</v>
       </c>
       <c r="AC4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD4">
         <v>0.2414</v>
@@ -1104,13 +1158,25 @@
         <v>1</v>
       </c>
       <c r="AK4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AM4">
         <v>0</v>
+      </c>
+      <c r="AN4">
+        <v>-0.61</v>
+      </c>
+      <c r="AO4">
+        <v>0.61</v>
+      </c>
+      <c r="AP4">
+        <v>-0.61</v>
+      </c>
+      <c r="AQ4">
+        <v>0.61</v>
       </c>
     </row>
     <row r="5" spans="1:43" x14ac:dyDescent="0.25">
@@ -1118,7 +1184,7 @@
         <v>43</v>
       </c>
       <c r="B5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C5">
         <v>4.5</v>
@@ -1132,26 +1198,32 @@
       <c r="F5">
         <v>5.24</v>
       </c>
+      <c r="G5">
+        <v>4</v>
+      </c>
       <c r="H5" t="s">
         <v>45</v>
       </c>
+      <c r="I5">
+        <v>0.74</v>
+      </c>
       <c r="J5" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="K5">
         <v>5.24</v>
       </c>
       <c r="L5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M5" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="N5">
         <v>824887</v>
       </c>
       <c r="O5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P5">
         <v>5.8</v>
@@ -1193,7 +1265,7 @@
         <v>1.1602</v>
       </c>
       <c r="AC5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD5">
         <v>0.258</v>
@@ -1217,13 +1289,25 @@
         <v>1</v>
       </c>
       <c r="AK5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AM5">
         <v>0</v>
+      </c>
+      <c r="AN5">
+        <v>-1.24</v>
+      </c>
+      <c r="AO5">
+        <v>1.24</v>
+      </c>
+      <c r="AP5">
+        <v>-1.24</v>
+      </c>
+      <c r="AQ5">
+        <v>1.24</v>
       </c>
     </row>
     <row r="6" spans="1:43" x14ac:dyDescent="0.25">
@@ -1231,7 +1315,7 @@
         <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C6">
         <v>4.5</v>
@@ -1245,26 +1329,32 @@
       <c r="F6">
         <v>3.88</v>
       </c>
+      <c r="G6">
+        <v>4</v>
+      </c>
       <c r="H6" t="s">
         <v>45</v>
       </c>
+      <c r="I6">
+        <v>-0.62</v>
+      </c>
       <c r="J6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K6">
         <v>3.88</v>
       </c>
       <c r="L6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M6" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="N6">
         <v>823675</v>
       </c>
       <c r="O6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P6">
         <v>5.5</v>
@@ -1306,7 +1396,7 @@
         <v>0.8374</v>
       </c>
       <c r="AC6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD6">
         <v>0.1862</v>
@@ -1330,13 +1420,25 @@
         <v>1</v>
       </c>
       <c r="AK6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AM6">
         <v>0</v>
+      </c>
+      <c r="AN6">
+        <v>0.12</v>
+      </c>
+      <c r="AO6">
+        <v>0.12</v>
+      </c>
+      <c r="AP6">
+        <v>0.12</v>
+      </c>
+      <c r="AQ6">
+        <v>0.12</v>
       </c>
     </row>
     <row r="7" spans="1:43" x14ac:dyDescent="0.25">
@@ -1344,7 +1446,7 @@
         <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C7">
         <v>5.5</v>
@@ -1358,26 +1460,32 @@
       <c r="F7">
         <v>6.3</v>
       </c>
+      <c r="G7">
+        <v>7</v>
+      </c>
       <c r="H7" t="s">
-        <v>45</v>
+        <v>54</v>
+      </c>
+      <c r="I7">
+        <v>0.8</v>
       </c>
       <c r="J7" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="K7">
         <v>6.3</v>
       </c>
       <c r="L7" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="M7" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="N7">
         <v>823675</v>
       </c>
       <c r="O7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P7">
         <v>5.1</v>
@@ -1419,7 +1527,7 @@
         <v>1.2887</v>
       </c>
       <c r="AC7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD7">
         <v>0.2866</v>
@@ -1443,13 +1551,25 @@
         <v>1</v>
       </c>
       <c r="AK7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AM7">
         <v>0</v>
+      </c>
+      <c r="AN7">
+        <v>0.7</v>
+      </c>
+      <c r="AO7">
+        <v>0.7</v>
+      </c>
+      <c r="AP7">
+        <v>0.7</v>
+      </c>
+      <c r="AQ7">
+        <v>0.7</v>
       </c>
     </row>
     <row r="8" spans="1:43" x14ac:dyDescent="0.25">
@@ -1457,7 +1577,7 @@
         <v>43</v>
       </c>
       <c r="B8" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C8">
         <v>3.5</v>
@@ -1471,26 +1591,32 @@
       <c r="F8">
         <v>3.41</v>
       </c>
+      <c r="G8">
+        <v>6</v>
+      </c>
       <c r="H8" t="s">
-        <v>45</v>
+        <v>54</v>
+      </c>
+      <c r="I8">
+        <v>-0.09</v>
       </c>
       <c r="J8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K8">
         <v>3.41</v>
       </c>
       <c r="L8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M8" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="N8">
         <v>823018</v>
       </c>
       <c r="O8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P8">
         <v>4.6</v>
@@ -1532,7 +1658,7 @@
         <v>0.9378</v>
       </c>
       <c r="AC8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD8">
         <v>0.2086</v>
@@ -1556,13 +1682,25 @@
         <v>1</v>
       </c>
       <c r="AK8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AM8">
         <v>0</v>
+      </c>
+      <c r="AN8">
+        <v>2.59</v>
+      </c>
+      <c r="AO8">
+        <v>2.59</v>
+      </c>
+      <c r="AP8">
+        <v>2.59</v>
+      </c>
+      <c r="AQ8">
+        <v>2.59</v>
       </c>
     </row>
     <row r="9" spans="1:43" x14ac:dyDescent="0.25">
@@ -1570,7 +1708,7 @@
         <v>43</v>
       </c>
       <c r="B9" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C9">
         <v>3.5</v>
@@ -1584,26 +1722,32 @@
       <c r="F9">
         <v>4.36</v>
       </c>
+      <c r="G9">
+        <v>6</v>
+      </c>
       <c r="H9" t="s">
-        <v>45</v>
+        <v>54</v>
+      </c>
+      <c r="I9">
+        <v>0.86</v>
       </c>
       <c r="J9" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="K9">
         <v>4.36</v>
       </c>
       <c r="L9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M9" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="N9">
         <v>823018</v>
       </c>
       <c r="O9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P9">
         <v>5.2</v>
@@ -1645,7 +1789,7 @@
         <v>0.998</v>
       </c>
       <c r="AC9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD9">
         <v>0.222</v>
@@ -1669,13 +1813,25 @@
         <v>1</v>
       </c>
       <c r="AK9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AM9">
         <v>0</v>
+      </c>
+      <c r="AN9">
+        <v>1.64</v>
+      </c>
+      <c r="AO9">
+        <v>1.64</v>
+      </c>
+      <c r="AP9">
+        <v>1.64</v>
+      </c>
+      <c r="AQ9">
+        <v>1.64</v>
       </c>
     </row>
     <row r="10" spans="1:43" x14ac:dyDescent="0.25">
@@ -1683,7 +1839,7 @@
         <v>43</v>
       </c>
       <c r="B10" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C10">
         <v>6.5</v>
@@ -1697,26 +1853,32 @@
       <c r="F10">
         <v>7.66</v>
       </c>
+      <c r="G10">
+        <v>9</v>
+      </c>
       <c r="H10" t="s">
-        <v>45</v>
+        <v>54</v>
+      </c>
+      <c r="I10">
+        <v>1.16</v>
       </c>
       <c r="J10" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="K10">
         <v>7.66</v>
       </c>
       <c r="L10" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="M10" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="N10">
         <v>823998</v>
       </c>
       <c r="O10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P10">
         <v>5.4</v>
@@ -1758,7 +1920,7 @@
         <v>1.2845</v>
       </c>
       <c r="AC10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD10">
         <v>0.2857</v>
@@ -1782,13 +1944,25 @@
         <v>1</v>
       </c>
       <c r="AK10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AM10">
         <v>0</v>
+      </c>
+      <c r="AN10">
+        <v>1.34</v>
+      </c>
+      <c r="AO10">
+        <v>1.34</v>
+      </c>
+      <c r="AP10">
+        <v>1.34</v>
+      </c>
+      <c r="AQ10">
+        <v>1.34</v>
       </c>
     </row>
     <row r="11" spans="1:43" x14ac:dyDescent="0.25">
@@ -1796,7 +1970,7 @@
         <v>43</v>
       </c>
       <c r="B11" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C11">
         <v>6.5</v>
@@ -1810,26 +1984,32 @@
       <c r="F11">
         <v>10.01</v>
       </c>
+      <c r="G11">
+        <v>6</v>
+      </c>
       <c r="H11" t="s">
         <v>45</v>
       </c>
+      <c r="I11">
+        <v>3.51</v>
+      </c>
       <c r="J11" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="K11">
         <v>10.01</v>
       </c>
       <c r="L11" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="M11" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="N11">
         <v>823998</v>
       </c>
       <c r="O11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P11">
         <v>5.6</v>
@@ -1871,7 +2051,7 @@
         <v>1.3326</v>
       </c>
       <c r="AC11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD11">
         <v>0.2964</v>
@@ -1895,13 +2075,25 @@
         <v>1</v>
       </c>
       <c r="AK11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AM11">
         <v>0</v>
+      </c>
+      <c r="AN11">
+        <v>-4.01</v>
+      </c>
+      <c r="AO11">
+        <v>4.01</v>
+      </c>
+      <c r="AP11">
+        <v>-4.01</v>
+      </c>
+      <c r="AQ11">
+        <v>4.01</v>
       </c>
     </row>
     <row r="12" spans="1:43" x14ac:dyDescent="0.25">
@@ -1909,7 +2101,7 @@
         <v>43</v>
       </c>
       <c r="B12" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C12">
         <v>3.5</v>
@@ -1923,26 +2115,32 @@
       <c r="F12">
         <v>3.98</v>
       </c>
+      <c r="G12">
+        <v>3</v>
+      </c>
       <c r="H12" t="s">
         <v>45</v>
       </c>
+      <c r="I12">
+        <v>0.48</v>
+      </c>
       <c r="J12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K12">
         <v>3.98</v>
       </c>
       <c r="L12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M12" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="N12">
         <v>825048</v>
       </c>
       <c r="O12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P12">
         <v>5.3</v>
@@ -1984,7 +2182,7 @@
         <v>0.8806</v>
       </c>
       <c r="AC12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD12">
         <v>0.1959</v>
@@ -2008,13 +2206,25 @@
         <v>1</v>
       </c>
       <c r="AK12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AM12">
         <v>0</v>
+      </c>
+      <c r="AN12">
+        <v>-0.98</v>
+      </c>
+      <c r="AO12">
+        <v>0.98</v>
+      </c>
+      <c r="AP12">
+        <v>-0.98</v>
+      </c>
+      <c r="AQ12">
+        <v>0.98</v>
       </c>
     </row>
     <row r="13" spans="1:43" x14ac:dyDescent="0.25">
@@ -2022,7 +2232,7 @@
         <v>43</v>
       </c>
       <c r="B13" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C13">
         <v>4.5</v>
@@ -2036,26 +2246,32 @@
       <c r="F13">
         <v>5.37</v>
       </c>
+      <c r="G13">
+        <v>4</v>
+      </c>
       <c r="H13" t="s">
         <v>45</v>
       </c>
+      <c r="I13">
+        <v>0.87</v>
+      </c>
       <c r="J13" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="K13">
         <v>5.37</v>
       </c>
       <c r="L13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M13" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="N13">
         <v>825048</v>
       </c>
       <c r="O13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P13">
         <v>5.5</v>
@@ -2097,7 +2313,7 @@
         <v>1.0394</v>
       </c>
       <c r="AC13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD13">
         <v>0.2312</v>
@@ -2121,13 +2337,25 @@
         <v>1</v>
       </c>
       <c r="AK13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AM13">
         <v>0</v>
+      </c>
+      <c r="AN13">
+        <v>-1.37</v>
+      </c>
+      <c r="AO13">
+        <v>1.37</v>
+      </c>
+      <c r="AP13">
+        <v>-1.37</v>
+      </c>
+      <c r="AQ13">
+        <v>1.37</v>
       </c>
     </row>
     <row r="14" spans="1:43" x14ac:dyDescent="0.25">
@@ -2135,7 +2363,7 @@
         <v>43</v>
       </c>
       <c r="B14" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C14">
         <v>4.5</v>
@@ -2149,26 +2377,32 @@
       <c r="F14">
         <v>4.63</v>
       </c>
+      <c r="G14">
+        <v>5</v>
+      </c>
       <c r="H14" t="s">
-        <v>45</v>
+        <v>54</v>
+      </c>
+      <c r="I14">
+        <v>0.13</v>
       </c>
       <c r="J14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K14">
         <v>4.63</v>
       </c>
       <c r="L14" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M14" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="N14">
         <v>824969</v>
       </c>
       <c r="O14" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P14">
         <v>5.1</v>
@@ -2210,7 +2444,7 @@
         <v>0.9274</v>
       </c>
       <c r="AC14" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD14">
         <v>0.2063</v>
@@ -2234,13 +2468,25 @@
         <v>1</v>
       </c>
       <c r="AK14" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL14" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AM14">
         <v>0</v>
+      </c>
+      <c r="AN14">
+        <v>0.37</v>
+      </c>
+      <c r="AO14">
+        <v>0.37</v>
+      </c>
+      <c r="AP14">
+        <v>0.37</v>
+      </c>
+      <c r="AQ14">
+        <v>0.37</v>
       </c>
     </row>
     <row r="15" spans="1:43" x14ac:dyDescent="0.25">
@@ -2248,7 +2494,7 @@
         <v>43</v>
       </c>
       <c r="B15" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C15">
         <v>4.5</v>
@@ -2262,26 +2508,32 @@
       <c r="F15">
         <v>3.36</v>
       </c>
+      <c r="G15">
+        <v>5</v>
+      </c>
       <c r="H15" t="s">
-        <v>45</v>
+        <v>54</v>
+      </c>
+      <c r="I15">
+        <v>-1.14</v>
       </c>
       <c r="J15" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="K15">
         <v>3.36</v>
       </c>
       <c r="L15" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M15" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="N15">
         <v>824969</v>
       </c>
       <c r="O15" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="P15">
         <v>4.4</v>
@@ -2323,7 +2575,7 @@
         <v>0.8052</v>
       </c>
       <c r="AC15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD15">
         <v>0.1791</v>
@@ -2347,13 +2599,25 @@
         <v>1</v>
       </c>
       <c r="AK15" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL15" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AM15">
         <v>0</v>
+      </c>
+      <c r="AN15">
+        <v>1.64</v>
+      </c>
+      <c r="AO15">
+        <v>1.64</v>
+      </c>
+      <c r="AP15">
+        <v>1.64</v>
+      </c>
+      <c r="AQ15">
+        <v>1.64</v>
       </c>
     </row>
     <row r="16" spans="1:43" x14ac:dyDescent="0.25">
@@ -2361,7 +2625,7 @@
         <v>43</v>
       </c>
       <c r="B16" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C16">
         <v>5.5</v>
@@ -2375,26 +2639,32 @@
       <c r="F16">
         <v>4.83</v>
       </c>
+      <c r="G16">
+        <v>7</v>
+      </c>
       <c r="H16" t="s">
-        <v>45</v>
+        <v>54</v>
+      </c>
+      <c r="I16">
+        <v>-0.67</v>
       </c>
       <c r="J16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K16">
         <v>4.83</v>
       </c>
       <c r="L16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M16" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="N16">
         <v>823265</v>
       </c>
       <c r="O16" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P16">
         <v>5</v>
@@ -2436,7 +2706,7 @@
         <v>0.7898</v>
       </c>
       <c r="AC16" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD16">
         <v>0.1757</v>
@@ -2460,13 +2730,25 @@
         <v>1</v>
       </c>
       <c r="AK16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AM16">
         <v>0</v>
+      </c>
+      <c r="AN16">
+        <v>2.17</v>
+      </c>
+      <c r="AO16">
+        <v>2.17</v>
+      </c>
+      <c r="AP16">
+        <v>2.17</v>
+      </c>
+      <c r="AQ16">
+        <v>2.17</v>
       </c>
     </row>
     <row r="17" spans="1:43" x14ac:dyDescent="0.25">
@@ -2474,7 +2756,7 @@
         <v>43</v>
       </c>
       <c r="B17" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C17">
         <v>4.5</v>
@@ -2488,26 +2770,32 @@
       <c r="F17">
         <v>4.95</v>
       </c>
+      <c r="G17">
+        <v>6</v>
+      </c>
       <c r="H17" t="s">
-        <v>45</v>
+        <v>54</v>
+      </c>
+      <c r="I17">
+        <v>0.45</v>
       </c>
       <c r="J17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K17">
         <v>4.95</v>
       </c>
       <c r="L17" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="N17">
         <v>823265</v>
       </c>
       <c r="O17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P17">
         <v>5.3</v>
@@ -2549,7 +2837,7 @@
         <v>1.0616</v>
       </c>
       <c r="AC17" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD17">
         <v>0.2361</v>
@@ -2573,13 +2861,25 @@
         <v>1</v>
       </c>
       <c r="AK17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AM17">
         <v>0</v>
+      </c>
+      <c r="AN17">
+        <v>1.05</v>
+      </c>
+      <c r="AO17">
+        <v>1.05</v>
+      </c>
+      <c r="AP17">
+        <v>1.05</v>
+      </c>
+      <c r="AQ17">
+        <v>1.05</v>
       </c>
     </row>
     <row r="18" spans="1:43" x14ac:dyDescent="0.25">
@@ -2587,7 +2887,7 @@
         <v>43</v>
       </c>
       <c r="B18" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C18">
         <v>3.5</v>
@@ -2601,26 +2901,32 @@
       <c r="F18">
         <v>3.66</v>
       </c>
+      <c r="G18">
+        <v>6</v>
+      </c>
       <c r="H18" t="s">
-        <v>45</v>
+        <v>54</v>
+      </c>
+      <c r="I18">
+        <v>0.16</v>
       </c>
       <c r="J18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K18">
         <v>3.66</v>
       </c>
       <c r="L18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M18" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N18">
         <v>823189</v>
       </c>
       <c r="O18" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P18">
         <v>5</v>
@@ -2662,7 +2968,7 @@
         <v>0.9308</v>
       </c>
       <c r="AC18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD18">
         <v>0.207</v>
@@ -2686,13 +2992,25 @@
         <v>1</v>
       </c>
       <c r="AK18" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL18" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AM18">
         <v>0</v>
+      </c>
+      <c r="AN18">
+        <v>2.34</v>
+      </c>
+      <c r="AO18">
+        <v>2.34</v>
+      </c>
+      <c r="AP18">
+        <v>2.34</v>
+      </c>
+      <c r="AQ18">
+        <v>2.34</v>
       </c>
     </row>
     <row r="19" spans="1:43" x14ac:dyDescent="0.25">
@@ -2700,7 +3018,7 @@
         <v>43</v>
       </c>
       <c r="B19" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C19">
         <v>4.5</v>
@@ -2714,26 +3032,32 @@
       <c r="F19">
         <v>4.92</v>
       </c>
+      <c r="G19">
+        <v>2</v>
+      </c>
       <c r="H19" t="s">
         <v>45</v>
       </c>
+      <c r="I19">
+        <v>0.42</v>
+      </c>
       <c r="J19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K19">
         <v>4.92</v>
       </c>
       <c r="L19" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M19" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="N19">
         <v>823918</v>
       </c>
       <c r="O19" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P19">
         <v>5.6</v>
@@ -2775,7 +3099,7 @@
         <v>0.9323</v>
       </c>
       <c r="AC19" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD19">
         <v>0.2074</v>
@@ -2799,13 +3123,25 @@
         <v>1</v>
       </c>
       <c r="AK19" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL19" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AM19">
         <v>0</v>
+      </c>
+      <c r="AN19">
+        <v>-2.92</v>
+      </c>
+      <c r="AO19">
+        <v>2.92</v>
+      </c>
+      <c r="AP19">
+        <v>-2.92</v>
+      </c>
+      <c r="AQ19">
+        <v>2.92</v>
       </c>
     </row>
     <row r="20" spans="1:43" x14ac:dyDescent="0.25">
@@ -2813,7 +3149,7 @@
         <v>43</v>
       </c>
       <c r="B20" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C20">
         <v>7.5</v>
@@ -2827,26 +3163,32 @@
       <c r="F20">
         <v>5.51</v>
       </c>
+      <c r="G20">
+        <v>6</v>
+      </c>
       <c r="H20" t="s">
         <v>45</v>
       </c>
+      <c r="I20">
+        <v>-1.99</v>
+      </c>
       <c r="J20" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="K20">
         <v>5.51</v>
       </c>
       <c r="L20" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M20" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="N20">
         <v>823918</v>
       </c>
       <c r="O20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P20">
         <v>6</v>
@@ -2888,7 +3230,7 @@
         <v>0.8243</v>
       </c>
       <c r="AC20" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AD20">
         <v>0.1833</v>
@@ -2912,13 +3254,25 @@
         <v>1</v>
       </c>
       <c r="AK20" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AL20" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AM20">
         <v>0</v>
+      </c>
+      <c r="AN20">
+        <v>0.49</v>
+      </c>
+      <c r="AO20">
+        <v>0.49</v>
+      </c>
+      <c r="AP20">
+        <v>0.49</v>
+      </c>
+      <c r="AQ20">
+        <v>0.49</v>
       </c>
     </row>
     <row r="21" spans="1:43" x14ac:dyDescent="0.25">
@@ -2926,7 +3280,7 @@
         <v>43</v>
       </c>
       <c r="B21" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C21">
         <v>3.5</v>
@@ -2937,38 +3291,41 @@
       <c r="E21">
         <v>134</v>
       </c>
+      <c r="G21">
+        <v>4</v>
+      </c>
       <c r="H21" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="J21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="L21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M21" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="S21">
         <v>6</v>
       </c>
       <c r="AC21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AK21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AL21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>